<commit_message>
LMDI: Legg til 100%-semantikk i beskrivelse av ProsentvisDoseendring
Tydeliggjør at en normal dose uten endring tilsvarer 100%, i tråd med
INSPIRE-spesifikasjonen. Formuleringen er harmonisert mellom extension-
beskrivelsen og definition-annotasjonen i Legemiddelrekvirering-profilen.

Closes #89 830268cde34d46ed06320c456f7d301786b5d69b
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-prosentvis-doseendring.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-prosentvis-doseendring.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-27T10:27:35+00:00</t>
+    <t>2026-04-07T13:07:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Doseendring i prosent, sammenlignet med opprinnelig dosering. Spesielt relevant ved kjemoterapi.</t>
+    <t>Doseendring i prosent, sammenlignet med opprinnelig dosering. Spesielt relevant ved kjemoterapi. En normal dose, uten modifiseringer, er 100%.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>